<commit_message>
Port figure 01 axis swap and simplify figure 14 to single-bar ΔATR
Headline revenue (fig 01): variant on x-axis, labor scenarios as the
colored fill (PAL_LABOR / "Labor scenario"). Foregrounds the growth-
magnitude comparison; labor is the secondary dimension.

ATR-by-decile (fig 14): drop the Extended-denominator bar pair; emit
a single YBL_BLUE bar per decile using the standard cf-pretax-income
denominator. Caption simplified to the standard ΔATR formula. Removes
the now-unused PAL_ATR_DEFN constant. 14b / 14c are unaffected.

Bundles + figure PNGs + figure_data_2030.xlsx regenerated from the
release sbatch (job 12892782, 10:28 elapsed).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/figures/2030/figure_data_2030.xlsx
+++ b/results/figures/2030/figure_data_2030.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="225">
   <si>
     <t xml:space="preserve">Title:</t>
   </si>
@@ -630,7 +630,7 @@
   </si>
   <si>
     <t xml:space="preserve">Source: The Budget Lab at Yale AI-Fiscal microsimulation model, FY 2030.
-Standard denominator = cf pretax income; Extended denominator = baseline pretax + gross factor expansion.
+ΔATR = (cf tax / cf pretax income) − (baseline tax / baseline pretax income).
 CIT omitted from denominator (consistent handling would require allocating CIT in baseline as well).</t>
   </si>
   <si>
@@ -655,13 +655,7 @@
     <t xml:space="preserve">atr_cf_std</t>
   </si>
   <si>
-    <t xml:space="preserve">atr_cf_ext</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dATR_std</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dATR_ext</t>
+    <t xml:space="preserve">dATR</t>
   </si>
   <si>
     <t xml:space="preserve">Slow shock, Compressive labor scenario (R, Mechanical), FY 2030</t>
@@ -697,9 +691,6 @@
     <t xml:space="preserve">Source: The Budget Lab at Yale AI-Fiscal microsimulation model, FY 2030.
 ΔATR = (cf tax / cf pretax income) − (baseline tax / baseline pretax income).
 Three bars per decile compare labor (inequality) scenarios at a fixed shock variant.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dATR</t>
   </si>
   <si>
     <t xml:space="preserve">1</t>
@@ -5556,8 +5547,6 @@
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5615,12 +5604,6 @@
       <c r="J5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -5651,13 +5634,7 @@
         <v>-0.0186684262458328</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0186940594228906</v>
-      </c>
-      <c r="K6" t="n">
         <v>0.0000511071166378642</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.0000254739395800681</v>
       </c>
     </row>
     <row r="7">
@@ -5689,13 +5666,7 @@
         <v>-0.0571721194798668</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0570905147651227</v>
-      </c>
-      <c r="K7" t="n">
         <v>-0.000133115586061432</v>
-      </c>
-      <c r="L7" t="n">
-        <v>-0.0000515108713172452</v>
       </c>
     </row>
     <row r="8">
@@ -5727,13 +5698,7 @@
         <v>-0.0506869239011938</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0506303169235891</v>
-      </c>
-      <c r="K8" t="n">
         <v>-0.000217735187236827</v>
-      </c>
-      <c r="L8" t="n">
-        <v>-0.000161128209632183</v>
       </c>
     </row>
     <row r="9">
@@ -5765,13 +5730,7 @@
         <v>-0.0147853178441947</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0147722117747558</v>
-      </c>
-      <c r="K9" t="n">
         <v>-0.000246250249430122</v>
-      </c>
-      <c r="L9" t="n">
-        <v>-0.000233144179991183</v>
       </c>
     </row>
     <row r="10">
@@ -5803,13 +5762,7 @@
         <v>0.0234768041516604</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0234551788969786</v>
-      </c>
-      <c r="K10" t="n">
         <v>-0.000216337746784225</v>
-      </c>
-      <c r="L10" t="n">
-        <v>-0.000237963001466047</v>
       </c>
     </row>
     <row r="11">
@@ -5841,13 +5794,7 @@
         <v>0.0486720657239264</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0486437528206063</v>
-      </c>
-      <c r="K11" t="n">
         <v>-0.0000655508587302303</v>
-      </c>
-      <c r="L11" t="n">
-        <v>-0.0000938637620503113</v>
       </c>
     </row>
     <row r="12">
@@ -5879,13 +5826,7 @@
         <v>0.0643745435798656</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0643435432044503</v>
-      </c>
-      <c r="K12" t="n">
         <v>-0.000074313261091502</v>
-      </c>
-      <c r="L12" t="n">
-        <v>-0.000105313636506774</v>
       </c>
     </row>
     <row r="13">
@@ -5917,13 +5858,7 @@
         <v>0.0800281887058866</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0799904179172678</v>
-      </c>
-      <c r="K13" t="n">
         <v>-0.0000282177186376187</v>
-      </c>
-      <c r="L13" t="n">
-        <v>-0.0000659885072564065</v>
       </c>
     </row>
     <row r="14">
@@ -5955,13 +5890,7 @@
         <v>0.106195080855864</v>
       </c>
       <c r="J14" t="n">
-        <v>0.10621382535286</v>
-      </c>
-      <c r="K14" t="n">
         <v>0.0000737413302169532</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.0000924858272128154</v>
       </c>
     </row>
     <row r="15">
@@ -5993,13 +5922,7 @@
         <v>0.185390495498426</v>
       </c>
       <c r="J15" t="n">
-        <v>0.185321610759645</v>
-      </c>
-      <c r="K15" t="n">
         <v>-0.0000319569404225728</v>
-      </c>
-      <c r="L15" t="n">
-        <v>-0.000100841679203517</v>
       </c>
     </row>
   </sheetData>
@@ -6023,8 +5946,6 @@
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6040,7 +5961,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3">
@@ -6082,12 +6003,6 @@
       <c r="J5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -6118,13 +6033,7 @@
         <v>-0.0184825980172762</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0185066217188571</v>
-      </c>
-      <c r="K6" t="n">
         <v>0.000236935345194454</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.00021291164361361</v>
       </c>
     </row>
     <row r="7">
@@ -6156,13 +6065,7 @@
         <v>-0.056521843292561</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0564510304224486</v>
-      </c>
-      <c r="K7" t="n">
         <v>0.000517160601244439</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.000587973471356772</v>
       </c>
     </row>
     <row r="8">
@@ -6194,13 +6097,7 @@
         <v>-0.0497526174223771</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0497064048288089</v>
-      </c>
-      <c r="K8" t="n">
         <v>0.000716571291579836</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.00076278388514802</v>
       </c>
     </row>
     <row r="9">
@@ -6232,13 +6129,7 @@
         <v>-0.0138249149461982</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0138146193324399</v>
-      </c>
-      <c r="K9" t="n">
         <v>0.000714152648566415</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.000724448262324708</v>
       </c>
     </row>
     <row r="10">
@@ -6270,13 +6161,7 @@
         <v>0.0242692043487644</v>
       </c>
       <c r="J10" t="n">
-        <v>0.024249363875287</v>
-      </c>
-      <c r="K10" t="n">
         <v>0.000576062450319745</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.000556221976842304</v>
       </c>
     </row>
     <row r="11">
@@ -6308,13 +6193,7 @@
         <v>0.0491153766734412</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0490907888079621</v>
-      </c>
-      <c r="K11" t="n">
         <v>0.000377760090784607</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.000353172225305537</v>
       </c>
     </row>
     <row r="12">
@@ -6346,13 +6225,7 @@
         <v>0.0647823916382626</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0647565250604146</v>
-      </c>
-      <c r="K12" t="n">
         <v>0.000333534797305537</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.000307668219457491</v>
       </c>
     </row>
     <row r="13">
@@ -6384,13 +6257,7 @@
         <v>0.080212975931865</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0801788587188638</v>
-      </c>
-      <c r="K13" t="n">
         <v>0.000156569507340817</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.000122452294339576</v>
       </c>
     </row>
     <row r="14">
@@ -6422,13 +6289,7 @@
         <v>0.106301170739188</v>
       </c>
       <c r="J14" t="n">
-        <v>0.106322755621391</v>
-      </c>
-      <c r="K14" t="n">
         <v>0.00017983121354026</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.000201416095743964</v>
       </c>
     </row>
     <row r="15">
@@ -6460,13 +6321,7 @@
         <v>0.184760356421856</v>
       </c>
       <c r="J15" t="n">
-        <v>0.184686056730729</v>
-      </c>
-      <c r="K15" t="n">
         <v>-0.00066209601699263</v>
-      </c>
-      <c r="L15" t="n">
-        <v>-0.000736395708120174</v>
       </c>
     </row>
   </sheetData>
@@ -6490,8 +6345,6 @@
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6507,7 +6360,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3">
@@ -6549,12 +6402,6 @@
       <c r="J5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -6585,13 +6432,7 @@
         <v>-0.0188544595662508</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0188817184378241</v>
-      </c>
-      <c r="K6" t="n">
         <v>-0.000134926203780139</v>
-      </c>
-      <c r="L6" t="n">
-        <v>-0.000162185075353379</v>
       </c>
     </row>
     <row r="7">
@@ -6623,13 +6464,7 @@
         <v>-0.0578039806568488</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0577112868954043</v>
-      </c>
-      <c r="K7" t="n">
         <v>-0.000764976763043379</v>
-      </c>
-      <c r="L7" t="n">
-        <v>-0.000672283001598883</v>
       </c>
     </row>
     <row r="8">
@@ -6661,13 +6496,7 @@
         <v>-0.0516116172058026</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.051544204742099</v>
-      </c>
-      <c r="K8" t="n">
         <v>-0.0011424284918457</v>
-      </c>
-      <c r="L8" t="n">
-        <v>-0.00107501602814204</v>
       </c>
     </row>
     <row r="9">
@@ -6699,13 +6528,7 @@
         <v>-0.015746602884162</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0157303949951399</v>
-      </c>
-      <c r="K9" t="n">
         <v>-0.00120753528939738</v>
-      </c>
-      <c r="L9" t="n">
-        <v>-0.00119132740037536</v>
       </c>
     </row>
     <row r="10">
@@ -6737,13 +6560,7 @@
         <v>0.0226740888071861</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0226508266257772</v>
-      </c>
-      <c r="K10" t="n">
         <v>-0.00101905309125856</v>
-      </c>
-      <c r="L10" t="n">
-        <v>-0.00104231527266744</v>
       </c>
     </row>
     <row r="11">
@@ -6775,13 +6592,7 @@
         <v>0.0482259007402664</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0481938893259736</v>
-      </c>
-      <c r="K11" t="n">
         <v>-0.000511715842390202</v>
-      </c>
-      <c r="L11" t="n">
-        <v>-0.000543727256682953</v>
       </c>
     </row>
     <row r="12">
@@ -6813,13 +6624,7 @@
         <v>0.0639609445220738</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0639248205689395</v>
-      </c>
-      <c r="K12" t="n">
         <v>-0.000487912318883274</v>
-      </c>
-      <c r="L12" t="n">
-        <v>-0.000524036272017581</v>
       </c>
     </row>
     <row r="13">
@@ -6851,13 +6656,7 @@
         <v>0.0798409448418348</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0797994791613741</v>
-      </c>
-      <c r="K13" t="n">
         <v>-0.000215461582689438</v>
-      </c>
-      <c r="L13" t="n">
-        <v>-0.000256927263150075</v>
       </c>
     </row>
     <row r="14">
@@ -6889,13 +6688,7 @@
         <v>0.106084856667424</v>
       </c>
       <c r="J14" t="n">
-        <v>0.106100702720218</v>
-      </c>
-      <c r="K14" t="n">
         <v>-0.0000364828582231636</v>
-      </c>
-      <c r="L14" t="n">
-        <v>-0.0000206368054298939</v>
       </c>
     </row>
     <row r="15">
@@ -6927,13 +6720,7 @@
         <v>0.186021340460792</v>
       </c>
       <c r="J15" t="n">
-        <v>0.185957907881391</v>
-      </c>
-      <c r="K15" t="n">
         <v>0.000598888021943689</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0.000535455442542659</v>
       </c>
     </row>
   </sheetData>
@@ -7554,8 +7341,6 @@
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7571,7 +7356,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3">
@@ -7613,12 +7398,6 @@
       <c r="J5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -7649,13 +7428,7 @@
         <v>-0.0189060485626329</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0190179838244689</v>
-      </c>
-      <c r="K6" t="n">
         <v>-0.000186515200162194</v>
-      </c>
-      <c r="L6" t="n">
-        <v>-0.000298450461998188</v>
       </c>
     </row>
     <row r="7">
@@ -7687,13 +7460,7 @@
         <v>-0.056771570539697</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0564313453961824</v>
-      </c>
-      <c r="K7" t="n">
         <v>0.000267433354108421</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.000607658497623023</v>
       </c>
     </row>
     <row r="8">
@@ -7725,13 +7492,7 @@
         <v>-0.0500414501314183</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0498117347991774</v>
-      </c>
-      <c r="K8" t="n">
         <v>0.000427738582538591</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.00065745391477956</v>
       </c>
     </row>
     <row r="9">
@@ -7763,13 +7524,7 @@
         <v>-0.0139061343994416</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0138557033252774</v>
-      </c>
-      <c r="K9" t="n">
         <v>0.000632933195322982</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.000683364269487148</v>
       </c>
     </row>
     <row r="10">
@@ -7801,13 +7556,7 @@
         <v>0.0243532271442149</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0242605743663021</v>
-      </c>
-      <c r="K10" t="n">
         <v>0.00066008524577028</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.000567432467857409</v>
       </c>
     </row>
     <row r="11">
@@ -7839,13 +7588,7 @@
         <v>0.0495500630599342</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0494345003618289</v>
-      </c>
-      <c r="K11" t="n">
         <v>0.000812446477277552</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.00069688377917234</v>
       </c>
     </row>
     <row r="12">
@@ -7877,13 +7620,7 @@
         <v>0.0653787721552891</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0652558058706256</v>
-      </c>
-      <c r="K12" t="n">
         <v>0.00092991531433205</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.000806949029668505</v>
       </c>
     </row>
     <row r="13">
@@ -7915,13 +7652,7 @@
         <v>0.0808255086531462</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0806747789929364</v>
-      </c>
-      <c r="K13" t="n">
         <v>0.000769102228622018</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.000618372568412212</v>
       </c>
     </row>
     <row r="14">
@@ -7953,13 +7684,7 @@
         <v>0.107613590108239</v>
       </c>
       <c r="J14" t="n">
-        <v>0.107713590954478</v>
-      </c>
-      <c r="K14" t="n">
         <v>0.00149225058259175</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.0015922514288305</v>
       </c>
     </row>
     <row r="15">
@@ -7991,13 +7716,7 @@
         <v>0.186505534592153</v>
       </c>
       <c r="J15" t="n">
-        <v>0.186234644204488</v>
-      </c>
-      <c r="K15" t="n">
         <v>0.00108308215330408</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0.00081219176563882</v>
       </c>
     </row>
   </sheetData>
@@ -8021,8 +7740,6 @@
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8038,7 +7755,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3">
@@ -8080,12 +7797,6 @@
       <c r="J5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -8116,13 +7827,7 @@
         <v>-0.0177711068626081</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0178690493135422</v>
-      </c>
-      <c r="K6" t="n">
         <v>0.000948426499862629</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.000850484048928488</v>
       </c>
     </row>
     <row r="7">
@@ -8154,13 +7859,7 @@
         <v>-0.0525543821726197</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0523061130498272</v>
-      </c>
-      <c r="K7" t="n">
         <v>0.00448462172118568</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.0047328908439782</v>
       </c>
     </row>
     <row r="8">
@@ -8192,13 +7891,7 @@
         <v>-0.0441342435419753</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0439887803846594</v>
-      </c>
-      <c r="K8" t="n">
         <v>0.00633494517198165</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.00648040832929752</v>
       </c>
     </row>
     <row r="9">
@@ -8230,13 +7923,7 @@
         <v>-0.008118392985046</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.00809663883806424</v>
-      </c>
-      <c r="K9" t="n">
         <v>0.00642067460971858</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.00644242875670034</v>
       </c>
     </row>
     <row r="10">
@@ -8268,13 +7955,7 @@
         <v>0.0289384180239176</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0288490414875068</v>
-      </c>
-      <c r="K10" t="n">
         <v>0.00524527612547299</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.00515589958906211</v>
       </c>
     </row>
     <row r="11">
@@ -8306,13 +7987,7 @@
         <v>0.0521909627012941</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0520968175520066</v>
-      </c>
-      <c r="K11" t="n">
         <v>0.00345334611863746</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.00335920096934999</v>
       </c>
     </row>
     <row r="12">
@@ -8344,13 +8019,7 @@
         <v>0.0677492855291876</v>
       </c>
       <c r="J12" t="n">
-        <v>0.067656964608825</v>
-      </c>
-      <c r="K12" t="n">
         <v>0.00330042868823052</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.00320810776786798</v>
       </c>
     </row>
     <row r="13">
@@ -8382,13 +8051,7 @@
         <v>0.0819110948512488</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0817823574624964</v>
-      </c>
-      <c r="K13" t="n">
         <v>0.00185468842672458</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.00172595103797218</v>
       </c>
     </row>
     <row r="14">
@@ -8420,13 +8083,7 @@
         <v>0.108186762150551</v>
       </c>
       <c r="J14" t="n">
-        <v>0.108303241950199</v>
-      </c>
-      <c r="K14" t="n">
         <v>0.00206542262490406</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.00218190242455177</v>
       </c>
     </row>
     <row r="15">
@@ -8458,13 +8115,7 @@
         <v>0.182754377325525</v>
       </c>
       <c r="J15" t="n">
-        <v>0.182450529346276</v>
-      </c>
-      <c r="K15" t="n">
         <v>-0.00266807511332401</v>
-      </c>
-      <c r="L15" t="n">
-        <v>-0.00297192309257269</v>
       </c>
     </row>
   </sheetData>
@@ -8488,8 +8139,6 @@
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8505,7 +8154,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3">
@@ -8547,12 +8196,6 @@
       <c r="J5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -8583,13 +8226,7 @@
         <v>-0.0200182447565166</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0201443409978793</v>
-      </c>
-      <c r="K6" t="n">
         <v>-0.00129871139404593</v>
-      </c>
-      <c r="L6" t="n">
-        <v>-0.00142480763540866</v>
       </c>
     </row>
     <row r="7">
@@ -8621,13 +8258,7 @@
         <v>-0.0602961180291157</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0598545788711062</v>
-      </c>
-      <c r="K7" t="n">
         <v>-0.00325711413531024</v>
-      </c>
-      <c r="L7" t="n">
-        <v>-0.00281557497730075</v>
       </c>
     </row>
     <row r="8">
@@ -8659,13 +8290,7 @@
         <v>-0.0555151199337701</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0551869538312763</v>
-      </c>
-      <c r="K8" t="n">
         <v>-0.00504593121981314</v>
-      </c>
-      <c r="L8" t="n">
-        <v>-0.00471776511731934</v>
       </c>
     </row>
     <row r="9">
@@ -8697,13 +8322,7 @@
         <v>-0.0197391180671867</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0196479134204269</v>
-      </c>
-      <c r="K9" t="n">
         <v>-0.00520005047242217</v>
-      </c>
-      <c r="L9" t="n">
-        <v>-0.00510884582566236</v>
       </c>
     </row>
     <row r="10">
@@ -8735,13 +8354,7 @@
         <v>0.0193667596627075</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0192782618854859</v>
-      </c>
-      <c r="K10" t="n">
         <v>-0.00432638223573716</v>
-      </c>
-      <c r="L10" t="n">
-        <v>-0.00441488001295876</v>
       </c>
     </row>
     <row r="11">
@@ -8773,13 +8386,7 @@
         <v>0.0468026943937539</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0466671433692886</v>
-      </c>
-      <c r="K11" t="n">
         <v>-0.00193492218890273</v>
-      </c>
-      <c r="L11" t="n">
-        <v>-0.00207047321336803</v>
       </c>
     </row>
     <row r="12">
@@ -8811,13 +8418,7 @@
         <v>0.0628208060454312</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0626680811804863</v>
-      </c>
-      <c r="K12" t="n">
         <v>-0.00162805079552591</v>
-      </c>
-      <c r="L12" t="n">
-        <v>-0.00178077566047075</v>
       </c>
     </row>
     <row r="13">
@@ -8849,13 +8450,7 @@
         <v>0.0796417939244897</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0794677276975093</v>
-      </c>
-      <c r="K13" t="n">
         <v>-0.000414612500034481</v>
-      </c>
-      <c r="L13" t="n">
-        <v>-0.000588678727014902</v>
       </c>
     </row>
     <row r="14">
@@ -8887,13 +8482,7 @@
         <v>0.106885545685425</v>
       </c>
       <c r="J14" t="n">
-        <v>0.106967057535163</v>
-      </c>
-      <c r="K14" t="n">
         <v>0.000764206159777486</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.000845718009515731</v>
       </c>
     </row>
     <row r="15">
@@ -8925,13 +8514,7 @@
         <v>0.190300194387076</v>
       </c>
       <c r="J15" t="n">
-        <v>0.190063651463431</v>
-      </c>
-      <c r="K15" t="n">
         <v>0.00487774194822752</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0.00464119902458246</v>
       </c>
     </row>
   </sheetData>
@@ -8955,8 +8538,6 @@
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8972,7 +8553,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3">
@@ -9014,12 +8595,6 @@
       <c r="J5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -9050,13 +8625,7 @@
         <v>-0.0187243193841494</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0189830176857129</v>
-      </c>
-      <c r="K6" t="n">
         <v>-0.00000478602167869324</v>
-      </c>
-      <c r="L6" t="n">
-        <v>-0.000263484323242205</v>
       </c>
     </row>
     <row r="7">
@@ -9088,13 +8657,7 @@
         <v>-0.0573160401390546</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0565177944691019</v>
-      </c>
-      <c r="K7" t="n">
         <v>-0.00027703624524919</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.000521209424703489</v>
       </c>
     </row>
     <row r="8">
@@ -9126,13 +8689,7 @@
         <v>-0.0509118442201434</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.050362828899998</v>
-      </c>
-      <c r="K8" t="n">
         <v>-0.00044265550618651</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.000106359813958935</v>
       </c>
     </row>
     <row r="9">
@@ -9164,13 +8721,7 @@
         <v>-0.0146745128062951</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0145493418248696</v>
-      </c>
-      <c r="K9" t="n">
         <v>-0.000135445211530508</v>
-      </c>
-      <c r="L9" t="n">
-        <v>-0.0000102742301050576</v>
       </c>
     </row>
     <row r="10">
@@ -9202,13 +8753,7 @@
         <v>0.0235981181088412</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0233879432166508</v>
-      </c>
-      <c r="K10" t="n">
         <v>-0.0000950237896034031</v>
-      </c>
-      <c r="L10" t="n">
-        <v>-0.000305198681793829</v>
       </c>
     </row>
     <row r="11">
@@ -9240,13 +8785,7 @@
         <v>0.0495448956744018</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0492717326064958</v>
-      </c>
-      <c r="K11" t="n">
         <v>0.000807279091745168</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.000534116023839189</v>
       </c>
     </row>
     <row r="12">
@@ -9278,13 +8817,7 @@
         <v>0.0652737517525397</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0649787152076434</v>
-      </c>
-      <c r="K12" t="n">
         <v>0.000824894911582677</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.000529858366686328</v>
       </c>
     </row>
     <row r="13">
@@ -9316,13 +8849,7 @@
         <v>0.0809975845290779</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0806375318275313</v>
-      </c>
-      <c r="K13" t="n">
         <v>0.000941178104553686</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.000581125403007074</v>
       </c>
     </row>
     <row r="14">
@@ -9354,13 +8881,7 @@
         <v>0.108411605299918</v>
       </c>
       <c r="J14" t="n">
-        <v>0.10862216801898</v>
-      </c>
-      <c r="K14" t="n">
         <v>0.00229026577427068</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.00250082849333255</v>
       </c>
     </row>
     <row r="15">
@@ -9392,13 +8913,7 @@
         <v>0.186766268219901</v>
       </c>
       <c r="J15" t="n">
-        <v>0.186139692500619</v>
-      </c>
-      <c r="K15" t="n">
         <v>0.00134381578105228</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0.000717240061770541</v>
       </c>
     </row>
   </sheetData>
@@ -9422,8 +8937,6 @@
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9439,7 +8952,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3">
@@ -9481,12 +8994,6 @@
       <c r="J5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -9517,13 +9024,7 @@
         <v>-0.0164902441731485</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0167075429192414</v>
-      </c>
-      <c r="K6" t="n">
         <v>0.00222928918932216</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.00201199044322931</v>
       </c>
     </row>
     <row r="7">
@@ -9555,13 +9056,7 @@
         <v>-0.0485565987977449</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0480370366394896</v>
-      </c>
-      <c r="K7" t="n">
         <v>0.00848240509606048</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.00900196725431578</v>
       </c>
     </row>
     <row r="8">
@@ -9593,13 +9088,7 @@
         <v>-0.0389192115498846</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0386144886088435</v>
-      </c>
-      <c r="K8" t="n">
         <v>0.0115499771640723</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.0118547001051134</v>
       </c>
     </row>
     <row r="9">
@@ -9631,13 +9120,7 @@
         <v>-0.00333217549236877</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.00331103322219745</v>
-      </c>
-      <c r="K9" t="n">
         <v>0.0112068921023958</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.0112280343725671</v>
       </c>
     </row>
     <row r="10">
@@ -9669,13 +9152,7 @@
         <v>0.0323805568378546</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0321481127670589</v>
-      </c>
-      <c r="K10" t="n">
         <v>0.00868741493940999</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.00845497086861427</v>
       </c>
     </row>
     <row r="11">
@@ -9707,13 +9184,7 @@
         <v>0.0546404008324257</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0544036922231216</v>
-      </c>
-      <c r="K11" t="n">
         <v>0.00590278424976909</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.00566607564046502</v>
       </c>
     </row>
     <row r="12">
@@ -9745,13 +9216,7 @@
         <v>0.0697675007205639</v>
       </c>
       <c r="J12" t="n">
-        <v>0.069529643690529</v>
-      </c>
-      <c r="K12" t="n">
         <v>0.00531864387960686</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.00508078684957189</v>
       </c>
     </row>
     <row r="13">
@@ -9783,13 +9248,7 @@
         <v>0.0830118727891467</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0826944864875204</v>
-      </c>
-      <c r="K13" t="n">
         <v>0.00295546636462247</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.00263808006299623</v>
       </c>
     </row>
     <row r="14">
@@ -9821,13 +9280,7 @@
         <v>0.109382795130369</v>
       </c>
       <c r="J14" t="n">
-        <v>0.109623833612075</v>
-      </c>
-      <c r="K14" t="n">
         <v>0.00326145560472128</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.00350249408642755</v>
       </c>
     </row>
     <row r="15">
@@ -9859,13 +9312,7 @@
         <v>0.179543192515306</v>
       </c>
       <c r="J15" t="n">
-        <v>0.178850388708376</v>
-      </c>
-      <c r="K15" t="n">
         <v>-0.00587925992354282</v>
-      </c>
-      <c r="L15" t="n">
-        <v>-0.00657206373047287</v>
       </c>
     </row>
   </sheetData>
@@ -9889,8 +9336,6 @@
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9906,7 +9351,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3">
@@ -9948,12 +9393,6 @@
       <c r="J5" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -9984,13 +9423,7 @@
         <v>-0.0209526291913949</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.0212537034929826</v>
-      </c>
-      <c r="K6" t="n">
         <v>-0.00223309582892427</v>
-      </c>
-      <c r="L6" t="n">
-        <v>-0.00253417013051193</v>
       </c>
     </row>
     <row r="7">
@@ -10022,13 +9455,7 @@
         <v>-0.0629135701699337</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0618151547351958</v>
-      </c>
-      <c r="K7" t="n">
         <v>-0.00587456627612826</v>
-      </c>
-      <c r="L7" t="n">
-        <v>-0.00477615084139039</v>
       </c>
     </row>
     <row r="8">
@@ -10060,13 +9487,7 @@
         <v>-0.0611550785961029</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.060299508154894</v>
-      </c>
-      <c r="K8" t="n">
         <v>-0.010685889882146</v>
-      </c>
-      <c r="L8" t="n">
-        <v>-0.00983031944093709</v>
       </c>
     </row>
     <row r="9">
@@ -10098,13 +9519,7 @@
         <v>-0.0260658322837742</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0257805292514384</v>
-      </c>
-      <c r="K9" t="n">
         <v>-0.0115267646890096</v>
-      </c>
-      <c r="L9" t="n">
-        <v>-0.0112414616566738</v>
       </c>
     </row>
     <row r="10">
@@ -10136,13 +9551,7 @@
         <v>0.0132726889304171</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0131282955227487</v>
-      </c>
-      <c r="K10" t="n">
         <v>-0.0104204529680275</v>
-      </c>
-      <c r="L10" t="n">
-        <v>-0.010564846375696</v>
       </c>
     </row>
     <row r="11">
@@ -10174,13 +9583,7 @@
         <v>0.0440153935299053</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0437134730326645</v>
-      </c>
-      <c r="K11" t="n">
         <v>-0.00472222305275127</v>
-      </c>
-      <c r="L11" t="n">
-        <v>-0.00502414354999212</v>
       </c>
     </row>
     <row r="12">
@@ -10212,13 +9615,7 @@
         <v>0.0600949150411036</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0597476624254135</v>
-      </c>
-      <c r="K12" t="n">
         <v>-0.00435394179985347</v>
-      </c>
-      <c r="L12" t="n">
-        <v>-0.0047011944155436</v>
       </c>
     </row>
     <row r="13">
@@ -10250,13 +9647,7 @@
         <v>0.0785724348164367</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0781642079985812</v>
-      </c>
-      <c r="K13" t="n">
         <v>-0.0014839716080875</v>
-      </c>
-      <c r="L13" t="n">
-        <v>-0.001892198425943</v>
       </c>
     </row>
     <row r="14">
@@ -10288,13 +9679,7 @@
         <v>0.106868915295283</v>
       </c>
       <c r="J14" t="n">
-        <v>0.107040944051524</v>
-      </c>
-      <c r="K14" t="n">
         <v>0.000747575769635411</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.000919604525876389</v>
       </c>
     </row>
     <row r="15">
@@ -10326,13 +9711,7 @@
         <v>0.194185682476493</v>
       </c>
       <c r="J15" t="n">
-        <v>0.193630497400647</v>
-      </c>
-      <c r="K15" t="n">
         <v>0.00876323003764432</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0.00820804496179842</v>
       </c>
     </row>
   </sheetData>
@@ -10367,7 +9746,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2">
@@ -10375,7 +9754,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3">
@@ -10383,7 +9762,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5">
@@ -10415,7 +9794,7 @@
         <v>195</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>9</v>
@@ -10435,7 +9814,7 @@
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C6" t="n">
         <v>-542.934369809947</v>
@@ -10479,7 +9858,7 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C7" t="n">
         <v>388.015540628305</v>
@@ -10523,7 +9902,7 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C8" t="n">
         <v>561.153333258383</v>
@@ -10567,7 +9946,7 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C9" t="n">
         <v>820.169437223817</v>
@@ -10611,7 +9990,7 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C10" t="n">
         <v>1092.09465240244</v>
@@ -10655,7 +10034,7 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C11" t="n">
         <v>1431.3633583382</v>
@@ -10699,7 +10078,7 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C12" t="n">
         <v>1878.29534636384</v>
@@ -10743,7 +10122,7 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C13" t="n">
         <v>2601.56180865961</v>
@@ -10787,7 +10166,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C14" t="n">
         <v>3791.68208048503</v>
@@ -10831,7 +10210,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C15" t="n">
         <v>11740.8308088609</v>
@@ -10875,7 +10254,7 @@
         <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C16" t="n">
         <v>-542.934369809947</v>
@@ -10919,7 +10298,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C17" t="n">
         <v>388.015540628305</v>
@@ -10963,7 +10342,7 @@
         <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C18" t="n">
         <v>561.153333258383</v>
@@ -11007,7 +10386,7 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C19" t="n">
         <v>820.169437223817</v>
@@ -11051,7 +10430,7 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C20" t="n">
         <v>1092.09465240244</v>
@@ -11095,7 +10474,7 @@
         <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C21" t="n">
         <v>1431.3633583382</v>
@@ -11139,7 +10518,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C22" t="n">
         <v>1878.29534636384</v>
@@ -11183,7 +10562,7 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C23" t="n">
         <v>2601.56180865961</v>
@@ -11227,7 +10606,7 @@
         <v>21</v>
       </c>
       <c r="B24" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C24" t="n">
         <v>3791.68208048503</v>
@@ -11271,7 +10650,7 @@
         <v>21</v>
       </c>
       <c r="B25" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C25" t="n">
         <v>11740.8308088609</v>
@@ -11315,7 +10694,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C26" t="n">
         <v>-542.934369809947</v>
@@ -11359,7 +10738,7 @@
         <v>24</v>
       </c>
       <c r="B27" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C27" t="n">
         <v>388.015540628305</v>
@@ -11403,7 +10782,7 @@
         <v>24</v>
       </c>
       <c r="B28" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C28" t="n">
         <v>561.153333258383</v>
@@ -11447,7 +10826,7 @@
         <v>24</v>
       </c>
       <c r="B29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C29" t="n">
         <v>820.169437223817</v>
@@ -11491,7 +10870,7 @@
         <v>24</v>
       </c>
       <c r="B30" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C30" t="n">
         <v>1092.09465240244</v>
@@ -11535,7 +10914,7 @@
         <v>24</v>
       </c>
       <c r="B31" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C31" t="n">
         <v>1431.3633583382</v>
@@ -11579,7 +10958,7 @@
         <v>24</v>
       </c>
       <c r="B32" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C32" t="n">
         <v>1878.29534636384</v>
@@ -11623,7 +11002,7 @@
         <v>24</v>
       </c>
       <c r="B33" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C33" t="n">
         <v>2601.56180865961</v>
@@ -11667,7 +11046,7 @@
         <v>24</v>
       </c>
       <c r="B34" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C34" t="n">
         <v>3791.68208048503</v>
@@ -11711,7 +11090,7 @@
         <v>24</v>
       </c>
       <c r="B35" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C35" t="n">
         <v>11740.8308088609</v>
@@ -11782,7 +11161,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2">
@@ -11790,7 +11169,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3">
@@ -11798,7 +11177,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5">
@@ -11830,7 +11209,7 @@
         <v>195</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>9</v>
@@ -11850,7 +11229,7 @@
         <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C6" t="n">
         <v>-542.934369809947</v>
@@ -11894,7 +11273,7 @@
         <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C7" t="n">
         <v>388.015540628305</v>
@@ -11938,7 +11317,7 @@
         <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C8" t="n">
         <v>561.153333258383</v>
@@ -11982,7 +11361,7 @@
         <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C9" t="n">
         <v>820.169437223817</v>
@@ -12026,7 +11405,7 @@
         <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C10" t="n">
         <v>1092.09465240244</v>
@@ -12070,7 +11449,7 @@
         <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C11" t="n">
         <v>1431.3633583382</v>
@@ -12114,7 +11493,7 @@
         <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C12" t="n">
         <v>1878.29534636384</v>
@@ -12158,7 +11537,7 @@
         <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C13" t="n">
         <v>2601.56180865961</v>
@@ -12202,7 +11581,7 @@
         <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C14" t="n">
         <v>3791.68208048503</v>
@@ -12246,7 +11625,7 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C15" t="n">
         <v>11740.8308088609</v>
@@ -12290,7 +11669,7 @@
         <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C16" t="n">
         <v>-542.934369809947</v>
@@ -12334,7 +11713,7 @@
         <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C17" t="n">
         <v>388.015540628305</v>
@@ -12378,7 +11757,7 @@
         <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C18" t="n">
         <v>561.153333258383</v>
@@ -12422,7 +11801,7 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C19" t="n">
         <v>820.169437223817</v>
@@ -12466,7 +11845,7 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C20" t="n">
         <v>1092.09465240244</v>
@@ -12510,7 +11889,7 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C21" t="n">
         <v>1431.3633583382</v>
@@ -12554,7 +11933,7 @@
         <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C22" t="n">
         <v>1878.29534636384</v>
@@ -12598,7 +11977,7 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C23" t="n">
         <v>2601.56180865961</v>
@@ -12642,7 +12021,7 @@
         <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C24" t="n">
         <v>3791.68208048503</v>
@@ -12686,7 +12065,7 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C25" t="n">
         <v>11740.8308088609</v>
@@ -12730,7 +12109,7 @@
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C26" t="n">
         <v>-542.934369809947</v>
@@ -12774,7 +12153,7 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C27" t="n">
         <v>388.015540628305</v>
@@ -12818,7 +12197,7 @@
         <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C28" t="n">
         <v>561.153333258383</v>
@@ -12862,7 +12241,7 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C29" t="n">
         <v>820.169437223817</v>
@@ -12906,7 +12285,7 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C30" t="n">
         <v>1092.09465240244</v>
@@ -12950,7 +12329,7 @@
         <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C31" t="n">
         <v>1431.3633583382</v>
@@ -12994,7 +12373,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C32" t="n">
         <v>1878.29534636384</v>
@@ -13038,7 +12417,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C33" t="n">
         <v>2601.56180865961</v>
@@ -13082,7 +12461,7 @@
         <v>31</v>
       </c>
       <c r="B34" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C34" t="n">
         <v>3791.68208048503</v>
@@ -13126,7 +12505,7 @@
         <v>31</v>
       </c>
       <c r="B35" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C35" t="n">
         <v>11740.8308088609</v>
@@ -13197,7 +12576,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2">
@@ -13205,7 +12584,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3">
@@ -13213,7 +12592,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5">
@@ -13245,7 +12624,7 @@
         <v>195</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>9</v>
@@ -13265,7 +12644,7 @@
         <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C6" t="n">
         <v>-542.934369809947</v>
@@ -13309,7 +12688,7 @@
         <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C7" t="n">
         <v>388.015540628305</v>
@@ -13353,7 +12732,7 @@
         <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C8" t="n">
         <v>561.153333258383</v>
@@ -13397,7 +12776,7 @@
         <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C9" t="n">
         <v>820.169437223817</v>
@@ -13441,7 +12820,7 @@
         <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C10" t="n">
         <v>1092.09465240244</v>
@@ -13485,7 +12864,7 @@
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C11" t="n">
         <v>1431.3633583382</v>
@@ -13529,7 +12908,7 @@
         <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C12" t="n">
         <v>1878.29534636384</v>
@@ -13573,7 +12952,7 @@
         <v>32</v>
       </c>
       <c r="B13" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C13" t="n">
         <v>2601.56180865961</v>
@@ -13617,7 +12996,7 @@
         <v>32</v>
       </c>
       <c r="B14" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C14" t="n">
         <v>3791.68208048503</v>
@@ -13661,7 +13040,7 @@
         <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C15" t="n">
         <v>11740.8308088609</v>
@@ -13705,7 +13084,7 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C16" t="n">
         <v>-542.934369809947</v>
@@ -13749,7 +13128,7 @@
         <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C17" t="n">
         <v>388.015540628305</v>
@@ -13793,7 +13172,7 @@
         <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C18" t="n">
         <v>561.153333258383</v>
@@ -13837,7 +13216,7 @@
         <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C19" t="n">
         <v>820.169437223817</v>
@@ -13881,7 +13260,7 @@
         <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C20" t="n">
         <v>1092.09465240244</v>
@@ -13925,7 +13304,7 @@
         <v>35</v>
       </c>
       <c r="B21" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C21" t="n">
         <v>1431.3633583382</v>
@@ -13969,7 +13348,7 @@
         <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C22" t="n">
         <v>1878.29534636384</v>
@@ -14013,7 +13392,7 @@
         <v>35</v>
       </c>
       <c r="B23" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C23" t="n">
         <v>2601.56180865961</v>
@@ -14057,7 +13436,7 @@
         <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C24" t="n">
         <v>3791.68208048503</v>
@@ -14101,7 +13480,7 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C25" t="n">
         <v>11740.8308088609</v>
@@ -14145,7 +13524,7 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C26" t="n">
         <v>-542.934369809947</v>
@@ -14189,7 +13568,7 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C27" t="n">
         <v>388.015540628305</v>
@@ -14233,7 +13612,7 @@
         <v>36</v>
       </c>
       <c r="B28" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C28" t="n">
         <v>561.153333258383</v>
@@ -14277,7 +13656,7 @@
         <v>36</v>
       </c>
       <c r="B29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C29" t="n">
         <v>820.169437223817</v>
@@ -14321,7 +13700,7 @@
         <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C30" t="n">
         <v>1092.09465240244</v>
@@ -14365,7 +13744,7 @@
         <v>36</v>
       </c>
       <c r="B31" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C31" t="n">
         <v>1431.3633583382</v>
@@ -14409,7 +13788,7 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C32" t="n">
         <v>1878.29534636384</v>
@@ -14453,7 +13832,7 @@
         <v>36</v>
       </c>
       <c r="B33" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C33" t="n">
         <v>2601.56180865961</v>
@@ -14497,7 +13876,7 @@
         <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C34" t="n">
         <v>3791.68208048503</v>
@@ -14541,7 +13920,7 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C35" t="n">
         <v>11740.8308088609</v>
@@ -14612,7 +13991,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2">
@@ -14620,7 +13999,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3">
@@ -14628,7 +14007,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
@@ -14660,7 +14039,7 @@
         <v>195</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>7</v>
@@ -14680,7 +14059,7 @@
         <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C6" t="n">
         <v>-542.934369809947</v>
@@ -14724,7 +14103,7 @@
         <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C7" t="n">
         <v>388.015540628305</v>
@@ -14768,7 +14147,7 @@
         <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C8" t="n">
         <v>561.153333258383</v>
@@ -14812,7 +14191,7 @@
         <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C9" t="n">
         <v>820.169437223817</v>
@@ -14856,7 +14235,7 @@
         <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C10" t="n">
         <v>1092.09465240244</v>
@@ -14900,7 +14279,7 @@
         <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C11" t="n">
         <v>1431.3633583382</v>
@@ -14944,7 +14323,7 @@
         <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C12" t="n">
         <v>1878.29534636384</v>
@@ -14988,7 +14367,7 @@
         <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C13" t="n">
         <v>2601.56180865961</v>
@@ -15032,7 +14411,7 @@
         <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C14" t="n">
         <v>3791.68208048503</v>
@@ -15076,7 +14455,7 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C15" t="n">
         <v>11740.8308088609</v>
@@ -15120,7 +14499,7 @@
         <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C16" t="n">
         <v>-542.934369809947</v>
@@ -15164,7 +14543,7 @@
         <v>32</v>
       </c>
       <c r="B17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C17" t="n">
         <v>388.015540628305</v>
@@ -15208,7 +14587,7 @@
         <v>32</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C18" t="n">
         <v>561.153333258383</v>
@@ -15252,7 +14631,7 @@
         <v>32</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C19" t="n">
         <v>820.169437223817</v>
@@ -15296,7 +14675,7 @@
         <v>32</v>
       </c>
       <c r="B20" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C20" t="n">
         <v>1092.09465240244</v>
@@ -15340,7 +14719,7 @@
         <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C21" t="n">
         <v>1431.3633583382</v>
@@ -15384,7 +14763,7 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C22" t="n">
         <v>1878.29534636384</v>
@@ -15428,7 +14807,7 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C23" t="n">
         <v>2601.56180865961</v>
@@ -15472,7 +14851,7 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C24" t="n">
         <v>3791.68208048503</v>
@@ -15516,7 +14895,7 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C25" t="n">
         <v>11740.8308088609</v>
@@ -15560,7 +14939,7 @@
         <v>14</v>
       </c>
       <c r="B26" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C26" t="n">
         <v>-542.934369809947</v>
@@ -15604,7 +14983,7 @@
         <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C27" t="n">
         <v>388.015540628305</v>
@@ -15648,7 +15027,7 @@
         <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C28" t="n">
         <v>561.153333258383</v>
@@ -15692,7 +15071,7 @@
         <v>14</v>
       </c>
       <c r="B29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C29" t="n">
         <v>820.169437223817</v>
@@ -15736,7 +15115,7 @@
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C30" t="n">
         <v>1092.09465240244</v>
@@ -15780,7 +15159,7 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C31" t="n">
         <v>1431.3633583382</v>
@@ -15824,7 +15203,7 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C32" t="n">
         <v>1878.29534636384</v>
@@ -15868,7 +15247,7 @@
         <v>14</v>
       </c>
       <c r="B33" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C33" t="n">
         <v>2601.56180865961</v>
@@ -15912,7 +15291,7 @@
         <v>14</v>
       </c>
       <c r="B34" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C34" t="n">
         <v>3791.68208048503</v>
@@ -15956,7 +15335,7 @@
         <v>14</v>
       </c>
       <c r="B35" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C35" t="n">
         <v>11740.8308088609</v>
@@ -17782,7 +17161,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2">
@@ -17790,7 +17169,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3">
@@ -17798,7 +17177,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
@@ -17830,7 +17209,7 @@
         <v>195</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>7</v>
@@ -17850,7 +17229,7 @@
         <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C6" t="n">
         <v>-542.934369809947</v>
@@ -17894,7 +17273,7 @@
         <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C7" t="n">
         <v>388.015540628305</v>
@@ -17938,7 +17317,7 @@
         <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C8" t="n">
         <v>561.153333258383</v>
@@ -17982,7 +17361,7 @@
         <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C9" t="n">
         <v>820.169437223817</v>
@@ -18026,7 +17405,7 @@
         <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C10" t="n">
         <v>1092.09465240244</v>
@@ -18070,7 +17449,7 @@
         <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C11" t="n">
         <v>1431.3633583382</v>
@@ -18114,7 +17493,7 @@
         <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C12" t="n">
         <v>1878.29534636384</v>
@@ -18158,7 +17537,7 @@
         <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C13" t="n">
         <v>2601.56180865961</v>
@@ -18202,7 +17581,7 @@
         <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C14" t="n">
         <v>3791.68208048503</v>
@@ -18246,7 +17625,7 @@
         <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C15" t="n">
         <v>11740.8308088609</v>
@@ -18290,7 +17669,7 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C16" t="n">
         <v>-542.934369809947</v>
@@ -18334,7 +17713,7 @@
         <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C17" t="n">
         <v>388.015540628305</v>
@@ -18378,7 +17757,7 @@
         <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C18" t="n">
         <v>561.153333258383</v>
@@ -18422,7 +17801,7 @@
         <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C19" t="n">
         <v>820.169437223817</v>
@@ -18466,7 +17845,7 @@
         <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C20" t="n">
         <v>1092.09465240244</v>
@@ -18510,7 +17889,7 @@
         <v>35</v>
       </c>
       <c r="B21" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C21" t="n">
         <v>1431.3633583382</v>
@@ -18554,7 +17933,7 @@
         <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C22" t="n">
         <v>1878.29534636384</v>
@@ -18598,7 +17977,7 @@
         <v>35</v>
       </c>
       <c r="B23" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C23" t="n">
         <v>2601.56180865961</v>
@@ -18642,7 +18021,7 @@
         <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C24" t="n">
         <v>3791.68208048503</v>
@@ -18686,7 +18065,7 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C25" t="n">
         <v>11740.8308088609</v>
@@ -18730,7 +18109,7 @@
         <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C26" t="n">
         <v>-542.934369809947</v>
@@ -18774,7 +18153,7 @@
         <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C27" t="n">
         <v>388.015540628305</v>
@@ -18818,7 +18197,7 @@
         <v>21</v>
       </c>
       <c r="B28" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C28" t="n">
         <v>561.153333258383</v>
@@ -18862,7 +18241,7 @@
         <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C29" t="n">
         <v>820.169437223817</v>
@@ -18906,7 +18285,7 @@
         <v>21</v>
       </c>
       <c r="B30" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C30" t="n">
         <v>1092.09465240244</v>
@@ -18950,7 +18329,7 @@
         <v>21</v>
       </c>
       <c r="B31" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C31" t="n">
         <v>1431.3633583382</v>
@@ -18994,7 +18373,7 @@
         <v>21</v>
       </c>
       <c r="B32" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C32" t="n">
         <v>1878.29534636384</v>
@@ -19038,7 +18417,7 @@
         <v>21</v>
       </c>
       <c r="B33" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C33" t="n">
         <v>2601.56180865961</v>
@@ -19082,7 +18461,7 @@
         <v>21</v>
       </c>
       <c r="B34" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C34" t="n">
         <v>3791.68208048503</v>
@@ -19126,7 +18505,7 @@
         <v>21</v>
       </c>
       <c r="B35" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C35" t="n">
         <v>11740.8308088609</v>
@@ -19197,7 +18576,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2">
@@ -19205,7 +18584,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3">
@@ -19213,7 +18592,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
@@ -19245,7 +18624,7 @@
         <v>195</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>7</v>
@@ -19265,7 +18644,7 @@
         <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C6" t="n">
         <v>-542.934369809947</v>
@@ -19309,7 +18688,7 @@
         <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C7" t="n">
         <v>388.015540628305</v>
@@ -19353,7 +18732,7 @@
         <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C8" t="n">
         <v>561.153333258383</v>
@@ -19397,7 +18776,7 @@
         <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C9" t="n">
         <v>820.169437223817</v>
@@ -19441,7 +18820,7 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C10" t="n">
         <v>1092.09465240244</v>
@@ -19485,7 +18864,7 @@
         <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C11" t="n">
         <v>1431.3633583382</v>
@@ -19529,7 +18908,7 @@
         <v>31</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C12" t="n">
         <v>1878.29534636384</v>
@@ -19573,7 +18952,7 @@
         <v>31</v>
       </c>
       <c r="B13" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C13" t="n">
         <v>2601.56180865961</v>
@@ -19617,7 +18996,7 @@
         <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C14" t="n">
         <v>3791.68208048503</v>
@@ -19661,7 +19040,7 @@
         <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C15" t="n">
         <v>11740.8308088609</v>
@@ -19705,7 +19084,7 @@
         <v>36</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C16" t="n">
         <v>-542.934369809947</v>
@@ -19749,7 +19128,7 @@
         <v>36</v>
       </c>
       <c r="B17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C17" t="n">
         <v>388.015540628305</v>
@@ -19793,7 +19172,7 @@
         <v>36</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C18" t="n">
         <v>561.153333258383</v>
@@ -19837,7 +19216,7 @@
         <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C19" t="n">
         <v>820.169437223817</v>
@@ -19881,7 +19260,7 @@
         <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C20" t="n">
         <v>1092.09465240244</v>
@@ -19925,7 +19304,7 @@
         <v>36</v>
       </c>
       <c r="B21" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C21" t="n">
         <v>1431.3633583382</v>
@@ -19969,7 +19348,7 @@
         <v>36</v>
       </c>
       <c r="B22" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C22" t="n">
         <v>1878.29534636384</v>
@@ -20013,7 +19392,7 @@
         <v>36</v>
       </c>
       <c r="B23" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C23" t="n">
         <v>2601.56180865961</v>
@@ -20057,7 +19436,7 @@
         <v>36</v>
       </c>
       <c r="B24" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C24" t="n">
         <v>3791.68208048503</v>
@@ -20101,7 +19480,7 @@
         <v>36</v>
       </c>
       <c r="B25" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C25" t="n">
         <v>11740.8308088609</v>
@@ -20145,7 +19524,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C26" t="n">
         <v>-542.934369809947</v>
@@ -20189,7 +19568,7 @@
         <v>24</v>
       </c>
       <c r="B27" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C27" t="n">
         <v>388.015540628305</v>
@@ -20233,7 +19612,7 @@
         <v>24</v>
       </c>
       <c r="B28" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C28" t="n">
         <v>561.153333258383</v>
@@ -20277,7 +19656,7 @@
         <v>24</v>
       </c>
       <c r="B29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C29" t="n">
         <v>820.169437223817</v>
@@ -20321,7 +19700,7 @@
         <v>24</v>
       </c>
       <c r="B30" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C30" t="n">
         <v>1092.09465240244</v>
@@ -20365,7 +19744,7 @@
         <v>24</v>
       </c>
       <c r="B31" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C31" t="n">
         <v>1431.3633583382</v>
@@ -20409,7 +19788,7 @@
         <v>24</v>
       </c>
       <c r="B32" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C32" t="n">
         <v>1878.29534636384</v>
@@ -20453,7 +19832,7 @@
         <v>24</v>
       </c>
       <c r="B33" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C33" t="n">
         <v>2601.56180865961</v>
@@ -20497,7 +19876,7 @@
         <v>24</v>
       </c>
       <c r="B34" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C34" t="n">
         <v>3791.68208048503</v>
@@ -20541,7 +19920,7 @@
         <v>24</v>
       </c>
       <c r="B35" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C35" t="n">
         <v>11740.8308088609</v>

</xml_diff>

<commit_message>
results: refresh 2030 bundles with decomposition levels (vintage 202607091035)
Re-run of the aggregation stage only (08/09) against the existing
Tax-Simulator output, to pick up the new baseline / counterfactual level
columns on the decomposition and synthetic grid rows.

No Tax-Simulator re-run: every delta in revenue_grid_long is identical
to the previous bundle to the last bit (234/234 rows, max absolute
difference 0). The workbooks gain columns, not numbers.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/figures/2030/figure_data_2030.xlsx
+++ b/results/figures/2030/figure_data_2030.xlsx
@@ -15504,8 +15504,12 @@
       <c r="J6" t="s">
         <v>54</v>
       </c>
-      <c r="K6"/>
-      <c r="L6"/>
+      <c r="K6" t="n">
+        <v>486.083</v>
+      </c>
+      <c r="L6" t="n">
+        <v>494.449322742468</v>
+      </c>
       <c r="M6" t="n">
         <v>8.36632274246801</v>
       </c>
@@ -15688,8 +15692,12 @@
       <c r="J10" t="s">
         <v>54</v>
       </c>
-      <c r="K10"/>
-      <c r="L10"/>
+      <c r="K10" t="n">
+        <v>486.083</v>
+      </c>
+      <c r="L10" t="n">
+        <v>494.449322742468</v>
+      </c>
       <c r="M10" t="n">
         <v>8.36632274246801</v>
       </c>
@@ -15872,8 +15880,12 @@
       <c r="J14" t="s">
         <v>54</v>
       </c>
-      <c r="K14"/>
-      <c r="L14"/>
+      <c r="K14" t="n">
+        <v>486.083</v>
+      </c>
+      <c r="L14" t="n">
+        <v>494.449322742468</v>
+      </c>
       <c r="M14" t="n">
         <v>8.36632274246801</v>
       </c>
@@ -16056,8 +16068,12 @@
       <c r="J18" t="s">
         <v>54</v>
       </c>
-      <c r="K18"/>
-      <c r="L18"/>
+      <c r="K18" t="n">
+        <v>486.083</v>
+      </c>
+      <c r="L18" t="n">
+        <v>522.741756959679</v>
+      </c>
       <c r="M18" t="n">
         <v>36.658756959679</v>
       </c>
@@ -16240,8 +16256,12 @@
       <c r="J22" t="s">
         <v>54</v>
       </c>
-      <c r="K22"/>
-      <c r="L22"/>
+      <c r="K22" t="n">
+        <v>486.083</v>
+      </c>
+      <c r="L22" t="n">
+        <v>522.741756959679</v>
+      </c>
       <c r="M22" t="n">
         <v>36.658756959679</v>
       </c>
@@ -16424,8 +16444,12 @@
       <c r="J26" t="s">
         <v>54</v>
       </c>
-      <c r="K26"/>
-      <c r="L26"/>
+      <c r="K26" t="n">
+        <v>486.083</v>
+      </c>
+      <c r="L26" t="n">
+        <v>522.741756959679</v>
+      </c>
       <c r="M26" t="n">
         <v>36.658756959679</v>
       </c>
@@ -16608,8 +16632,12 @@
       <c r="J30" t="s">
         <v>54</v>
       </c>
-      <c r="K30"/>
-      <c r="L30"/>
+      <c r="K30" t="n">
+        <v>486.083</v>
+      </c>
+      <c r="L30" t="n">
+        <v>570.084171098744</v>
+      </c>
       <c r="M30" t="n">
         <v>84.0011710987443</v>
       </c>
@@ -16792,8 +16820,12 @@
       <c r="J34" t="s">
         <v>54</v>
       </c>
-      <c r="K34"/>
-      <c r="L34"/>
+      <c r="K34" t="n">
+        <v>486.083</v>
+      </c>
+      <c r="L34" t="n">
+        <v>570.084171098744</v>
+      </c>
       <c r="M34" t="n">
         <v>84.0011710987443</v>
       </c>
@@ -16976,8 +17008,12 @@
       <c r="J38" t="s">
         <v>54</v>
       </c>
-      <c r="K38"/>
-      <c r="L38"/>
+      <c r="K38" t="n">
+        <v>486.083</v>
+      </c>
+      <c r="L38" t="n">
+        <v>570.084171098744</v>
+      </c>
       <c r="M38" t="n">
         <v>84.0011710987443</v>
       </c>

</xml_diff>